<commit_message>
Added saving tool and a RAG option to the runners.
</commit_message>
<xml_diff>
--- a/benchmark_runs/agent_evals_humaneval.xlsx
+++ b/benchmark_runs/agent_evals_humaneval.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mesfinbt/src/dissertation/read-mas/benchmark_runs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CB05304-9DE3-C648-93D6-F8AEFB902FBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05770C47-373F-4644-AB98-2B3102B9ACB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="41120" windowHeight="25780" activeTab="1" xr2:uid="{4F0CE36D-3AD7-B041-B516-82B89A187357}"/>
   </bookViews>
@@ -558,6 +558,12 @@
       <c r="B2">
         <v>0.92100000000000004</v>
       </c>
+      <c r="C2">
+        <v>0.872</v>
+      </c>
+      <c r="D2">
+        <v>0.84799999999999998</v>
+      </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -565,6 +571,12 @@
       </c>
       <c r="B3">
         <v>0.86599999999999999</v>
+      </c>
+      <c r="C3">
+        <v>0.82899999999999996</v>
+      </c>
+      <c r="D3">
+        <v>0.78400000000000003</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
@@ -671,6 +683,12 @@
       <c r="B6">
         <v>0.92100000000000004</v>
       </c>
+      <c r="C6">
+        <v>0.872</v>
+      </c>
+      <c r="D6">
+        <v>0.84799999999999998</v>
+      </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -678,6 +696,12 @@
       </c>
       <c r="B7">
         <v>0.86599999999999999</v>
+      </c>
+      <c r="C7">
+        <v>0.82899999999999996</v>
+      </c>
+      <c r="D7">
+        <v>0.78400000000000003</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added an overall wrapper agent to the orchestrator.
</commit_message>
<xml_diff>
--- a/benchmark_runs/agent_evals_humaneval.xlsx
+++ b/benchmark_runs/agent_evals_humaneval.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mesfinbt/src/dissertation/read-mas/benchmark_runs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05770C47-373F-4644-AB98-2B3102B9ACB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E07DDD8F-A804-0341-AAC2-4E3887596738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="41120" windowHeight="25780" activeTab="1" xr2:uid="{4F0CE36D-3AD7-B041-B516-82B89A187357}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="24">
   <si>
     <t>Model</t>
   </si>
@@ -599,68 +599,77 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6344593E-61CA-DC47-B2D2-E4019142A1A6}">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5" customWidth="1"/>
+    <col min="2" max="3" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1">
+      <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1">
         <v>1</v>
       </c>
-      <c r="D1" s="2">
+      <c r="E1" s="2">
         <v>2</v>
       </c>
-      <c r="E1" s="1">
+      <c r="F1" s="1">
         <v>3</v>
       </c>
-      <c r="F1" s="1">
+      <c r="G1" s="1">
         <v>4</v>
       </c>
-      <c r="G1" s="1">
+      <c r="H1" s="1">
         <v>5</v>
       </c>
-      <c r="H1" s="1">
+      <c r="I1" s="1">
         <v>6</v>
       </c>
-      <c r="I1" s="1">
+      <c r="J1" s="1">
         <v>7</v>
       </c>
-      <c r="J1" s="1">
+      <c r="K1" s="1">
         <v>8</v>
       </c>
-      <c r="K1" s="1">
+      <c r="L1" s="1">
         <v>9</v>
       </c>
-      <c r="L1" s="1">
+      <c r="M1" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
       <c r="B2">
         <v>0.64</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="C2">
+        <v>0.82299999999999995</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>11</v>
       </c>
       <c r="B3">
         <v>0.57899999999999996</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="C3">
+        <v>0.77400000000000002</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -668,7 +677,7 @@
         <v>0.73199999999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -676,57 +685,57 @@
         <v>0.65900000000000003</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>3</v>
       </c>
       <c r="B6">
         <v>0.92100000000000004</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>0.872</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>0.84799999999999998</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
       <c r="B7">
         <v>0.86599999999999999</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>0.82899999999999996</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>0.78400000000000003</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>23</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D1" r:id="rId1" display="Pass@1" xr:uid="{84DD76B2-3F57-4649-A89F-00D016702EBB}"/>
+    <hyperlink ref="E1" r:id="rId1" display="Pass@1" xr:uid="{84DD76B2-3F57-4649-A89F-00D016702EBB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added agent and models callbacks for debugging.
</commit_message>
<xml_diff>
--- a/benchmark_runs/agent_evals_humaneval.xlsx
+++ b/benchmark_runs/agent_evals_humaneval.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mesfinbt/src/dissertation/read-mas/benchmark_runs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E07DDD8F-A804-0341-AAC2-4E3887596738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC913659-C2A0-E641-B090-A82F27F5928A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="41120" windowHeight="25780" activeTab="1" xr2:uid="{4F0CE36D-3AD7-B041-B516-82B89A187357}"/>
   </bookViews>
@@ -666,7 +666,7 @@
         <v>0.57899999999999996</v>
       </c>
       <c r="C3">
-        <v>0.77400000000000002</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">

</xml_diff>